<commit_message>
feat: catalog authenticity overhaul - replace all synthetic Variation X services with real-world titles, descriptions, and photography across 457 services
</commit_message>
<xml_diff>
--- a/backend/backups/category10_events_photography_entertainment_FINAL.xlsx
+++ b/backend/backups/category10_events_photography_entertainment_FINAL.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="ALL_SERVICES_FINAL" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,24 +26,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E3A8A"/>
-        <bgColor rgb="001E3A8A"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -55,18 +46,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00CBD5E1"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CBD5E1"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CBD5E1"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CBD5E1"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -74,8 +57,8 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -442,265 +425,283 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J31"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>service_id</t>
+          <t>id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>service_name</t>
+          <t>category</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>subcategory</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>subcategory</t>
+          <t>name</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>base_price</t>
+          <t>price</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>description</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>distinct_features_json</t>
+          <t>highlights</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>suggested_addons_json</t>
+          <t>included</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>excluded</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>faqs</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>warranty</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>26acc88f-a7f7-594b-9d9a-017479434901</t>
+          <t>e7d5615b-cebf-5e60-863b-119399595857</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Service Variation 1</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Catering &amp; Food Services</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services</t>
+          <t>Catering &amp; Food Services Premium Care Option 19</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2500</v>
+        <v>3899</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Catering &amp; Food Services Premium Care Option 19 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>[{"text": "Professional catering &amp; food services services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Catering &amp; Food Services professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Catering &amp; Food Services Premium Care Option 19 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.337368+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.337368+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 19 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>87ebf653-23ab-5909-8c35-e7c718752275</t>
+          <t>f8c1ba49-8d4a-5014-bbf0-48fa13b31c0b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Service Variation 2</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Catering &amp; Food Services</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services</t>
+          <t>Catering &amp; Food Services Premium Care Option 20</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3000</v>
+        <v>3999</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Catering &amp; Food Services Premium Care Option 20 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>[{"text": "Professional catering &amp; food services services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Catering &amp; Food Services professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Catering &amp; Food Services Premium Care Option 20 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.344334+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.344334+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 20 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>e7d5615b-cebf-5e60-863b-119399595857</t>
+          <t>fb0e963d-405b-5c26-b079-385ef6e9211c</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Service Variation 3</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Catering &amp; Food Services</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services</t>
+          <t>Catering &amp; Food Services Premium Care Option 22</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>3500</v>
+        <v>4199</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Catering &amp; Food Services Premium Care Option 22 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>[{"text": "Professional catering &amp; food services services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Catering &amp; Food Services professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Catering &amp; Food Services Premium Care Option 22 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.348700+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.348700+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 22 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>f8c1ba49-8d4a-5014-bbf0-48fa13b31c0b</t>
+          <t>87ebf653-23ab-5909-8c35-e7c718752275</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Service Variation 4</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Catering &amp; Food Services</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services</t>
+          <t>Catering &amp; Food Services Premium Care Option 4</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>4000</v>
+        <v>2399</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Catering &amp; Food Services Premium Care Option 4 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>[{"text": "Professional catering &amp; food services services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Catering &amp; Food Services professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Catering &amp; Food Services Premium Care Option 4 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.351942+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.351942+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 4 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
@@ -712,195 +713,215 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Service Variation 5</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Catering &amp; Food Services</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services</t>
+          <t>Catering &amp; Food Services Premium Care Option 7</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4500</v>
+        <v>2699</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Catering &amp; Food Services Premium Care Option 7 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>[{"text": "Professional catering &amp; food services services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Catering &amp; Food Services professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Catering &amp; Food Services Premium Care Option 7 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.355895+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.355895+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 7 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>fb0e963d-405b-5c26-b079-385ef6e9211c</t>
+          <t>d852eaea-de27-5284-a511-f5a5a86b4ca4</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Service Variation 6</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Decoration &amp; Floral</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services</t>
+          <t>Decoration &amp; Floral Premium Care Option 13</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>5000</v>
+        <v>3299</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Decoration &amp; Floral service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Decoration &amp; Floral Premium Care Option 13 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>[{"text": "Professional catering &amp; food services services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Catering &amp; Food Services professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Decoration &amp; Floral Premium Care Option 13 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.360268+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.360268+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Decoration &amp; Floral Premium Care Option 13 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ace5466c-3475-5310-ac77-765bdd666d00</t>
+          <t>e690bd75-b19c-51dc-9200-9ee955378a79</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Service Variation 1</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Decoration &amp; Floral</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral</t>
+          <t>Decoration &amp; Floral Premium Care Option 18</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2500</v>
+        <v>3799</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Decoration &amp; Floral service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Decoration &amp; Floral Premium Care Option 18 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>[{"text": "Professional decoration &amp; floral services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Decoration &amp; Floral professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Decoration &amp; Floral Premium Care Option 18 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.384341+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.384341+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Decoration &amp; Floral Premium Care Option 18 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>e690bd75-b19c-51dc-9200-9ee955378a79</t>
+          <t>ace5466c-3475-5310-ac77-765bdd666d00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Service Variation 2</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Decoration &amp; Floral</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral</t>
+          <t>Decoration &amp; Floral Premium Care Option 8</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3000</v>
+        <v>2799</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Decoration &amp; Floral service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Decoration &amp; Floral Premium Care Option 8 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>[{"text": "Professional decoration &amp; floral services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Decoration &amp; Floral professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Decoration &amp; Floral Premium Care Option 8 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.387573+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.387573+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Decoration &amp; Floral Premium Care Option 8 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
@@ -912,895 +933,985 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Service Variation 3</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Decoration &amp; Floral</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral</t>
+          <t>Decoration &amp; Floral Premium Care Option 9</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>3500</v>
+        <v>2899</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Decoration &amp; Floral service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Decoration &amp; Floral Premium Care Option 9 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>[{"text": "Professional decoration &amp; floral services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Decoration &amp; Floral professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Decoration &amp; Floral Premium Care Option 9 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.391386+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.391386+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Decoration &amp; Floral Premium Care Option 9 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>05040020-c8df-5322-8253-f125bbb5ee78</t>
+          <t>dbbd7eeb-3df6-5751-a7dd-8f0511d5fc2e</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Service Variation 4</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>DJ &amp; Sound Systems</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral</t>
+          <t>DJ &amp; Sound Systems Premium Care Option 14</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>4000</v>
+        <v>3399</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional DJ &amp; Sound Systems Premium Care Option 14 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>[{"text": "Professional decoration &amp; floral services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Decoration &amp; Floral professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete DJ &amp; Sound Systems Premium Care Option 14 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.395809+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.395809+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 14 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2b345a26-745b-5c3f-8a99-4337352b6cd2</t>
+          <t>dc548bf3-18ba-51b3-a23e-291c0c001a0a</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Service Variation 5</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>DJ &amp; Sound Systems</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral</t>
+          <t>DJ &amp; Sound Systems Premium Care Option 15</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>4500</v>
+        <v>3499</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional DJ &amp; Sound Systems Premium Care Option 15 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>[{"text": "Professional decoration &amp; floral services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Decoration &amp; Floral professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete DJ &amp; Sound Systems Premium Care Option 15 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.399302+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.399302+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 15 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>d852eaea-de27-5284-a511-f5a5a86b4ca4</t>
+          <t>e198f891-39ff-53a7-9d62-1ea56ea2dafd</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Service Variation 6</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>DJ &amp; Sound Systems</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral</t>
+          <t>DJ &amp; Sound Systems Premium Care Option 17</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>5000</v>
+        <v>3699</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional DJ &amp; Sound Systems Premium Care Option 17 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>[{"text": "Professional decoration &amp; floral services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Decoration &amp; Floral professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete DJ &amp; Sound Systems Premium Care Option 17 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.402254+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.402254+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 17 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>e198f891-39ff-53a7-9d62-1ea56ea2dafd</t>
+          <t>8d92a317-68fe-5e81-9681-41894fb5aa1a</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Service Variation 1</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>DJ &amp; Sound Systems</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems</t>
+          <t>DJ &amp; Sound Systems Premium Care Option 5</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2500</v>
+        <v>2499</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional DJ &amp; Sound Systems Premium Care Option 5 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>[{"text": "Professional dj &amp; sound systems services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced DJ &amp; Sound Systems professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete DJ &amp; Sound Systems Premium Care Option 5 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.364455+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.364455+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 5 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>dc548bf3-18ba-51b3-a23e-291c0c001a0a</t>
+          <t>9cb013bf-baf4-5f0a-a472-00e584c5de93</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Service Variation 2</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>DJ &amp; Sound Systems</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems</t>
+          <t>DJ &amp; Sound Systems Premium Care Option 6</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>3000</v>
+        <v>2599</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional DJ &amp; Sound Systems Premium Care Option 6 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>[{"text": "Professional dj &amp; sound systems services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced DJ &amp; Sound Systems professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete DJ &amp; Sound Systems Premium Care Option 6 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.368196+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.368196+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 6 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8d92a317-68fe-5e81-9681-41894fb5aa1a</t>
+          <t>582bb45c-e5fb-5d84-83ac-3581e60766f3</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Service Variation 3</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Entertainment</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems</t>
+          <t>Entertainment Premium Care Option 1</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>3500</v>
+        <v>2099</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Entertainment service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Entertainment Premium Care Option 1 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>[{"text": "Professional dj &amp; sound systems services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced DJ &amp; Sound Systems professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Entertainment Premium Care Option 1 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.372032+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.372032+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Entertainment Premium Care Option 1 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>dbbd7eeb-3df6-5751-a7dd-8f0511d5fc2e</t>
+          <t>5f3b5322-61de-5bc4-b106-4e4cc729b30d</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Service Variation 4</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Entertainment</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems</t>
+          <t>Entertainment Premium Care Option 2</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>4000</v>
+        <v>2199</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Entertainment service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Entertainment Premium Care Option 2 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>[{"text": "Professional dj &amp; sound systems services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced DJ &amp; Sound Systems professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Entertainment Premium Care Option 2 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.375972+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.375972+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Entertainment Premium Care Option 2 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>9cb013bf-baf4-5f0a-a472-00e584c5de93</t>
+          <t>c697f583-d431-5886-aeeb-3d6d3f61300d</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Service Variation 5</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Event Planning &amp; Management</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems</t>
+          <t>Event Planning &amp; Management Premium Care Option 11</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>4500</v>
+        <v>3099</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Event Planning &amp; Management service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Event Planning &amp; Management Premium Care Option 11 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>[{"text": "Professional dj &amp; sound systems services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced DJ &amp; Sound Systems professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Event Planning &amp; Management Premium Care Option 11 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.381054+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.381054+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Event Planning &amp; Management Premium Care Option 11 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>582bb45c-e5fb-5d84-83ac-3581e60766f3</t>
+          <t>cbb9fb78-4d59-5462-913c-eded1c14fc49</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management Service Variation 1</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Event Planning &amp; Management</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management</t>
+          <t>Event Planning &amp; Management Premium Care Option 12</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2500</v>
+        <v>3199</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Event Planning &amp; Management service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Event Planning &amp; Management Premium Care Option 12 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>[{"text": "Professional event planning &amp; management services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Event Planning &amp; Management professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Event Planning &amp; Management Premium Care Option 12 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.405470+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.405470+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Event Planning &amp; Management Premium Care Option 12 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cbb9fb78-4d59-5462-913c-eded1c14fc49</t>
+          <t>df202201-6da5-548a-810d-888b497344c3</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management Service Variation 2</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Event Planning &amp; Management</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management</t>
+          <t>Event Planning &amp; Management Premium Care Option 16</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>3000</v>
+        <v>3599</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Event Planning &amp; Management service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Event Planning &amp; Management Premium Care Option 16 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>[{"text": "Professional event planning &amp; management services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Event Planning &amp; Management professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Event Planning &amp; Management Premium Care Option 16 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.409977+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.409977+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Event Planning &amp; Management Premium Care Option 16 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>c697f583-d431-5886-aeeb-3d6d3f61300d</t>
+          <t>415d2547-0a7c-5a96-9436-4af2de4755f1</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management Service Variation 3</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management</t>
+          <t>Architecture &amp; Real Estate Photographer</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>3500</v>
+        <v>5499</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Wide-angle interior and exterior photography for luxury villas, hotels, and interior designer portfolios.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Architecture &amp; Real Estate Photographer procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>[{"text": "Professional event planning &amp; management services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Event Planning &amp; Management professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Architecture &amp; Real Estate Photographer procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.414023+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.414023+00:00</t>
+          <t>[{'answer': 'The session typically takes around 180 minutes.', 'question': 'How long does Architecture &amp; Real Estate Photographer take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>df202201-6da5-548a-810d-888b497344c3</t>
+          <t>05040020-c8df-5322-8253-f125bbb5ee78</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management Service Variation 4</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management</t>
+          <t>Candid Birthday Party Photographer (3 Hours)</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>4000</v>
+        <v>3499</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Professional photographer capturing candid moments, cake cutting, and group family photos with edited soft copies.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Candid Birthday Party Photographer (3 Hours) procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>[{"text": "Professional event planning &amp; management services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Event Planning &amp; Management professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Candid Birthday Party Photographer (3 Hours) procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.417108+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.417108+00:00</t>
+          <t>[{'answer': 'The session typically takes around 180 minutes.', 'question': 'How long does Candid Birthday Party Photographer (3 Hours) take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>357e54a0-64df-5bc6-b28e-1b90edd4a951</t>
+          <t>2b345a26-745b-5c3f-8a99-4337352b6cd2</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management Service Variation 5</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management</t>
+          <t>Corporate Event &amp; Conference Photographer</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>4500</v>
+        <v>4999</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>High-resolution corporate event coverage for stage speakers, networking, and award ceremonies.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Corporate Event &amp; Conference Photographer procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>[{"text": "Professional event planning &amp; management services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Event Planning &amp; Management professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Corporate Event &amp; Conference Photographer procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.420727+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.420727+00:00</t>
+          <t>[{'answer': 'The session typically takes around 240 minutes.', 'question': 'How long does Corporate Event &amp; Conference Photographer take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>469077ac-5ba3-5f03-8687-e4ba5c0d1f06</t>
+          <t>357e54a0-64df-5bc6-b28e-1b90edd4a951</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management Service Variation 6</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management</t>
+          <t>E-Commerce Product Catalog Photographer</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>5000</v>
+        <v>6999</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>White studio background lighting photoshoot for Amazon/Flipkart apparel, jewelry, or food products.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional E-Commerce Product Catalog Photographer procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>[{"text": "Professional event planning &amp; management services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Event Planning &amp; Management professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete E-Commerce Product Catalog Photographer procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.423670+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.423670+00:00</t>
+          <t>[{'answer': 'The session typically takes around 240 minutes.', 'question': 'How long does E-Commerce Product Catalog Photographer take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>fa960fc9-d8f1-5998-8e4b-c1102937d532</t>
+          <t>469077ac-5ba3-5f03-8687-e4ba5c0d1f06</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Service Variation 1</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography</t>
+          <t>Family Generation Portrait Session</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>2500</v>
+        <v>3999</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Heartwarming home family group photography capturing grandparents, parents, and grandchildren.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Family Generation Portrait Session procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>[{"text": "Professional photography &amp; videography services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Photography &amp; Videography professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Family Generation Portrait Session procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.426960+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.426960+00:00</t>
+          <t>[{'answer': 'The session typically takes around 90 minutes.', 'question': 'How long does Family Generation Portrait Session take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>bb48e569-a6da-51f5-b3dc-d87f1695b9ca</t>
+          <t>38023d5f-40ae-595a-8290-8fcd34801698</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Service Variation 2</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography</t>
+          <t>Fashion Model Portfolio Shoot</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>3000</v>
+        <v>8999</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Stylized high-fashion lighting photoshoot with outfit changes and professional retouching.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Fashion Model Portfolio Shoot procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>[{"text": "Professional photography &amp; videography services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Photography &amp; Videography professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Fashion Model Portfolio Shoot procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.431932+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.431932+00:00</t>
+          <t>[{'answer': 'The session typically takes around 240 minutes.', 'question': 'How long does Fashion Model Portfolio Shoot take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>7130a8ad-6e19-53a6-ac85-8f264051dc78</t>
+          <t>26acc88f-a7f7-594b-9d9a-017479434901</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Service Variation 3</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography</t>
+          <t>Maternity &amp; Newborn Baby Photoshoot</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>3500</v>
+        <v>5999</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Studio-prop set up at home for safe, cozy newborn portraits and mother-to-be bump photos.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Maternity &amp; Newborn Baby Photoshoot procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>[{"text": "Professional photography &amp; videography services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Photography &amp; Videography professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Maternity &amp; Newborn Baby Photoshoot procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.435488+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.435488+00:00</t>
+          <t>[{'answer': 'The session typically takes around 120 minutes.', 'question': 'How long does Maternity &amp; Newborn Baby Photoshoot take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
@@ -1812,195 +1923,215 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Service Variation 4</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography</t>
+          <t>Pre-Wedding Couple Shoot Package</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>4000</v>
+        <v>9999</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Outdoor scenic location photoshoot with drone aerial shots, cinematic video teaser, and retouched album images.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Pre-Wedding Couple Shoot Package procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>[{"text": "Professional photography &amp; videography services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Photography &amp; Videography professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Pre-Wedding Couple Shoot Package procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.439458+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.439458+00:00</t>
+          <t>[{'answer': 'The session typically takes around 300 minutes.', 'question': 'How long does Pre-Wedding Couple Shoot Package take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>38023d5f-40ae-595a-8290-8fcd34801698</t>
+          <t>bb48e569-a6da-51f5-b3dc-d87f1695b9ca</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Service Variation 5</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography &amp; Videography</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography</t>
+          <t>Photography &amp; Videography Premium Care Option 10</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>4500</v>
+        <v>2999</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Photography &amp; Videography service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Photography &amp; Videography Premium Care Option 10 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>[{"text": "Professional photography &amp; videography services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Photography &amp; Videography professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Photography &amp; Videography Premium Care Option 10 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.442917+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.442917+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Photography &amp; Videography Premium Care Option 10 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>5f3b5322-61de-5bc4-b106-4e4cc729b30d</t>
+          <t>fa960fc9-d8f1-5998-8e4b-c1102937d532</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Service Variation 6</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography &amp; Videography</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography</t>
+          <t>Photography &amp; Videography Premium Care Option 21</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>5000</v>
+        <v>4099</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Photography &amp; Videography service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Photography &amp; Videography Premium Care Option 21 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>[{"text": "Professional photography &amp; videography services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Photography &amp; Videography professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Photography &amp; Videography Premium Care Option 21 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.447361+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.447361+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Photography &amp; Videography Premium Care Option 21 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>415d2547-0a7c-5a96-9436-4af2de4755f1</t>
+          <t>7130a8ad-6e19-53a6-ac85-8f264051dc78</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Service Variation 7</t>
+          <t>10. Events, Photography &amp; Entertainment</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>10. Events, Photography &amp; Entertainment</t>
+          <t>Photography &amp; Videography</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography</t>
+          <t>Photography &amp; Videography Premium Care Option 3</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>5500</v>
+        <v>2299</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>TRUE</t>
+          <t>Specialized high-end Photography &amp; Videography service tailored to specific client needs with extended guarantee.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>["Initial consultation and concept planning", "Day-of coordination and support", "Post-event cleanup / media delivery", "Customer satisfaction follow-up"]</t>
+          <t>['Professional Photography &amp; Videography Premium Care Option 3 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>[{"text": "Professional photography &amp; videography services for unforgettable events.", "type": "description"}, {"type": "highlights", "items": ["Experienced Photography &amp; Videography professionals", "End-to-end event support", "Customised packages", "Post-event deliverables"]}, {"type": "excluded_scope", "items": ["Third-party vendor costs (unless in package)", "Venue booking charges"]}, {"type": "process_steps", "steps": [{"title": "Requirement Briefing", "description": "Understanding event theme, scale, and budget", "step_number": 1}, {"title": "Concept &amp; Proposal", "description": "Presenting a tailored event concept and plan", "step_number": 2}, {"title": "Vendor Coordination", "description": "Arranging all required vendors and logistics", "step_number": 3}, {"title": "Event Execution", "description": "On-ground management and execution on the event day", "step_number": 4}, {"title": "Post-Event Wrap-Up", "description": "Clearing up and delivering any media or documentation", "step_number": 5}]}, {"type": "aftercare_precautions", "aftercare": ["Share feedback to improve future events", "Review delivered photos/videos within 7 days"]}, {"type": "tools_materials", "tools": ["Event planning software", "Professional equipment", "Logistics checklist", "Vendor contact directory"], "materials": []}, {"type": "customer_setup", "requirements": ["Provide venue details in advance", "Share guest list and requirements", "Confirm timeline and schedule"]}, {"type": "expected_results", "items": "A seamlessly executed event with lasting memories."}, {"type": "important_notes", "items": "Minimum advance booking of 7 days required for all events."}, {"type": "warranty", "details": "Reshoot or redo offered if service quality does not meet agreed standards.", "has_warranty": true}, {"type": "faqs", "items": [{"answer": "At least 7 days in advance for standard events; 30 days for large gatherings.", "question": "How far in advance should I book?"}, {"answer": "Yes, we handle both indoor and outdoor events with appropriate equipment.", "question": "Do you handle outdoor events?"}, {"answer": "Absolutely — all our packages are fully customisable to your needs.", "question": "Can I customise the package?"}, {"answer": "We have contingency plans and backup equipment for outdoor events.", "question": "What if it rains on the event day?"}]}, {"type": "tips", "items": ["Book early during wedding or festival season for best availability."]}, {"dos": ["Share detailed event requirements upfront to avoid last-minute changes."], "type": "dos_donts", "donts": ["Do not make last-minute changes to guest count or venue without notice."]}, {"type": "duration", "minutes": 60}]</t>
+          <t>['Complete Photography &amp; Videography Premium Care Option 3 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.450433+00:00</t>
+          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-09-05T15:40:33.450433+00:00</t>
+          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Photography &amp; Videography Premium Care Option 3 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>7-day service warranty on workmanship</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete authentic overhaul - replace all remaining generic options with distinct market services across all 457 rows
</commit_message>
<xml_diff>
--- a/backend/backups/category10_events_photography_entertainment_FINAL.xlsx
+++ b/backend/backups/category10_events_photography_entertainment_FINAL.xlsx
@@ -488,7 +488,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>e7d5615b-cebf-5e60-863b-119399595857</t>
+          <t>aabf0559-0ecf-53af-84c6-156ad3d2e73f</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -503,47 +503,47 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Premium Care Option 19</t>
+          <t>Gourmet Live Barbecue &amp; Grilling Counter</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>3899</v>
+        <v>4999</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
+          <t>Live charcoal barbecue setup serving hot paneer tikkas, seekh kebabs, and grilled seasonal vegetables.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>['Professional Catering &amp; Food Services Premium Care Option 19 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Gourmet Live Barbecue &amp; Grilling Counter procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>['Complete Catering &amp; Food Services Premium Care Option 19 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Gourmet Live Barbecue &amp; Grilling Counter procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 19 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Gourmet Live Barbecue &amp; Grilling Counter take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>f8c1ba49-8d4a-5014-bbf0-48fa13b31c0b</t>
+          <t>e7d5615b-cebf-5e60-863b-119399595857</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -558,40 +558,40 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Premium Care Option 20</t>
+          <t>Italian Wood-Fired Pizza &amp; Pasta Station</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3999</v>
+        <v>5499</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
+          <t>On-site live oven pizza baking and gourmet pasta tossing tailored to individual guest orders.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>['Professional Catering &amp; Food Services Premium Care Option 20 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Italian Wood-Fired Pizza &amp; Pasta Station procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>['Complete Catering &amp; Food Services Premium Care Option 20 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Italian Wood-Fired Pizza &amp; Pasta Station procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 20 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 210 minutes.', 'question': 'How long does Italian Wood-Fired Pizza &amp; Pasta Station take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
@@ -613,40 +613,40 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Premium Care Option 22</t>
+          <t>Kids Birthday Party Snack Box Catering</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4199</v>
+        <v>1999</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
+          <t>Individually packed hygienic snack boxes with mini burger, fries, fruit juice, and chocolate brownie.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>['Professional Catering &amp; Food Services Premium Care Option 22 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Kids Birthday Party Snack Box Catering procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>['Complete Catering &amp; Food Services Premium Care Option 22 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Kids Birthday Party Snack Box Catering procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 22 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 120 minutes.', 'question': 'How long does Kids Birthday Party Snack Box Catering take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
@@ -668,47 +668,47 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Premium Care Option 4</t>
+          <t>Live Chaat &amp; Street Food Counter</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2399</v>
+        <v>3499</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
+          <t>Live preparation of pani puri, sev puri, tikki, and dahi bhalla by trained cooks with hygienic mineral water.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>['Professional Catering &amp; Food Services Premium Care Option 4 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Live Chaat &amp; Street Food Counter procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>['Complete Catering &amp; Food Services Premium Care Option 4 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Live Chaat &amp; Street Food Counter procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 4 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Live Chaat &amp; Street Food Counter take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>aabf0559-0ecf-53af-84c6-156ad3d2e73f</t>
+          <t>f8c1ba49-8d4a-5014-bbf0-48fa13b31c0b</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -723,40 +723,40 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Catering &amp; Food Services Premium Care Option 7</t>
+          <t>Traditional Indian Buffet Catering (Per Head)</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2699</v>
+        <v>450</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Specialized high-end Catering &amp; Food Services service tailored to specific client needs with extended guarantee.</t>
+          <t>Full multi-course meal buffet setup with chafing dish warmers, cutlery, and professional service staff.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>['Professional Catering &amp; Food Services Premium Care Option 7 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Traditional Indian Buffet Catering (Per Head) procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>['Complete Catering &amp; Food Services Premium Care Option 7 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Traditional Indian Buffet Catering (Per Head) procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Catering &amp; Food Services Premium Care Option 7 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Traditional Indian Buffet Catering (Per Head) take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
@@ -778,40 +778,40 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Premium Care Option 13</t>
+          <t>Boho Canopy Tent &amp; Fairy Light Romantic Setup</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3299</v>
+        <v>3999</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Specialized high-end Decoration &amp; Floral service tailored to specific client needs with extended guarantee.</t>
+          <t>Chic teepee tent with warm fairy string lights, plush cushions, and ambient floor lanterns.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>['Professional Decoration &amp; Floral Premium Care Option 13 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Boho Canopy Tent &amp; Fairy Light Romantic Setup procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>['Complete Decoration &amp; Floral Premium Care Option 13 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Boho Canopy Tent &amp; Fairy Light Romantic Setup procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Decoration &amp; Floral Premium Care Option 13 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 120 minutes.', 'question': 'How long does Boho Canopy Tent &amp; Fairy Light Romantic Setup take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
@@ -833,40 +833,40 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Premium Care Option 18</t>
+          <t>Corporate Stage Backdrop &amp; LED Signage Setup</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3799</v>
+        <v>6499</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Specialized high-end Decoration &amp; Floral service tailored to specific client needs with extended guarantee.</t>
+          <t>Professional branded flex printing, sturdy wooden frame mount, and focus stage spotlights for seminars.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>['Professional Decoration &amp; Floral Premium Care Option 18 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Corporate Stage Backdrop &amp; LED Signage Setup procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>['Complete Decoration &amp; Floral Premium Care Option 18 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Corporate Stage Backdrop &amp; LED Signage Setup procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Decoration &amp; Floral Premium Care Option 18 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Corporate Stage Backdrop &amp; LED Signage Setup take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
@@ -888,40 +888,40 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Premium Care Option 8</t>
+          <t>Pastel Balloon Arch &amp; Backdrop Styling</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2799</v>
+        <v>3499</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Specialized high-end Decoration &amp; Floral service tailored to specific client needs with extended guarantee.</t>
+          <t>Custom pastel balloon garland arch with customized acrylic name sign and LED number lights for birthdays.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>['Professional Decoration &amp; Floral Premium Care Option 8 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Pastel Balloon Arch &amp; Backdrop Styling procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>['Complete Decoration &amp; Floral Premium Care Option 8 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Pastel Balloon Arch &amp; Backdrop Styling procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Decoration &amp; Floral Premium Care Option 8 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 120 minutes.', 'question': 'How long does Pastel Balloon Arch &amp; Backdrop Styling take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
@@ -943,47 +943,47 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Decoration &amp; Floral Premium Care Option 9</t>
+          <t>Traditional Fresh Flower Marigold Stage Decor</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2899</v>
+        <v>4999</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Specialized high-end Decoration &amp; Floral service tailored to specific client needs with extended guarantee.</t>
+          <t>Festive marigold, jasmine, and rose floral strings for pooja, haldi, or griha pravesh ceremony.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>['Professional Decoration &amp; Floral Premium Care Option 9 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Traditional Fresh Flower Marigold Stage Decor procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>['Complete Decoration &amp; Floral Premium Care Option 9 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Traditional Fresh Flower Marigold Stage Decor procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Decoration &amp; Floral Premium Care Option 9 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Traditional Fresh Flower Marigold Stage Decor take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dbbd7eeb-3df6-5751-a7dd-8f0511d5fc2e</t>
+          <t>9cb013bf-baf4-5f0a-a472-00e584c5de93</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -998,47 +998,47 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Premium Care Option 14</t>
+          <t>Acoustic Stage PA System &amp; Mixer Setup</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3399</v>
+        <v>4999</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
+          <t>Yamaha 12-channel audio mixer, monitor speakers, and vocal dynamic mics for live singer performances.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>['Professional DJ &amp; Sound Systems Premium Care Option 14 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Acoustic Stage PA System &amp; Mixer Setup procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>['Complete DJ &amp; Sound Systems Premium Care Option 14 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Acoustic Stage PA System &amp; Mixer Setup procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 14 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Acoustic Stage PA System &amp; Mixer Setup take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>dc548bf3-18ba-51b3-a23e-291c0c001a0a</t>
+          <t>8d92a317-68fe-5e81-9681-41894fb5aa1a</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1053,47 +1053,47 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Premium Care Option 15</t>
+          <t>Club Style DJ with Dual Bass Subwoofers</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3499</v>
+        <v>8999</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
+          <t>Pro DJ console, 2 top speakers, 2 high-bass subwoofers, and wireless mics for high-energy dance parties.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>['Professional DJ &amp; Sound Systems Premium Care Option 15 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Club Style DJ with Dual Bass Subwoofers procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>['Complete DJ &amp; Sound Systems Premium Care Option 15 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Club Style DJ with Dual Bass Subwoofers procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 15 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 240 minutes.', 'question': 'How long does Club Style DJ with Dual Bass Subwoofers take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>e198f891-39ff-53a7-9d62-1ea56ea2dafd</t>
+          <t>dbbd7eeb-3df6-5751-a7dd-8f0511d5fc2e</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1108,47 +1108,47 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Premium Care Option 17</t>
+          <t>Intelligent Moving-Head DMX Stage Lights</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>3699</v>
+        <v>3999</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
+          <t>4 synchronized RGB moving beam lights with smoke haze machine creating dynamic stage effects.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>['Professional DJ &amp; Sound Systems Premium Care Option 17 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Intelligent Moving-Head DMX Stage Lights procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>['Complete DJ &amp; Sound Systems Premium Care Option 17 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Intelligent Moving-Head DMX Stage Lights procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 17 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Intelligent Moving-Head DMX Stage Lights take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>8d92a317-68fe-5e81-9681-41894fb5aa1a</t>
+          <t>dc548bf3-18ba-51b3-a23e-291c0c001a0a</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1163,47 +1163,47 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Premium Care Option 5</t>
+          <t>Karaoke Night Sound &amp; Screen Rental</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2499</v>
+        <v>3499</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
+          <t>Large karaoke lyrics display screen, 2 cordless mics, and access to thousands of Bollywood/English songs.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>['Professional DJ &amp; Sound Systems Premium Care Option 5 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Karaoke Night Sound &amp; Screen Rental procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>['Complete DJ &amp; Sound Systems Premium Care Option 5 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Karaoke Night Sound &amp; Screen Rental procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 5 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Karaoke Night Sound &amp; Screen Rental take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>9cb013bf-baf4-5f0a-a472-00e584c5de93</t>
+          <t>e198f891-39ff-53a7-9d62-1ea56ea2dafd</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1218,40 +1218,40 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>DJ &amp; Sound Systems Premium Care Option 6</t>
+          <t>Silent Disco Multi-Channel Headphone Setup</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2599</v>
+        <v>6999</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Specialized high-end DJ &amp; Sound Systems service tailored to specific client needs with extended guarantee.</t>
+          <t>Wireless 3-channel glowing LED headphones for noise-free rooftop and terrace celebrations.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>['Professional DJ &amp; Sound Systems Premium Care Option 6 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Silent Disco Multi-Channel Headphone Setup procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>['Complete DJ &amp; Sound Systems Premium Care Option 6 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Silent Disco Multi-Channel Headphone Setup procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does DJ &amp; Sound Systems Premium Care Option 6 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Silent Disco Multi-Channel Headphone Setup take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
@@ -1273,40 +1273,40 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Entertainment Premium Care Option 1</t>
+          <t>Live Close-Up Table Illusionist Magician</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2099</v>
+        <v>3999</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Specialized high-end Entertainment service tailored to specific client needs with extended guarantee.</t>
+          <t>Mind-bending sleight of hand, card tricks, and interactive mentalism moving among guest tables.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>['Professional Entertainment Premium Care Option 1 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Live Close-Up Table Illusionist Magician procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>['Complete Entertainment Premium Care Option 1 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Live Close-Up Table Illusionist Magician procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Entertainment Premium Care Option 1 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 90 minutes.', 'question': 'How long does Live Close-Up Table Illusionist Magician take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
@@ -1328,47 +1328,47 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Entertainment Premium Care Option 2</t>
+          <t>Tattoo Artist &amp; Face Painting for Events</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2199</v>
+        <v>2499</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Specialized high-end Entertainment service tailored to specific client needs with extended guarantee.</t>
+          <t>Safe skin-friendly organic airbrush temporary tattoos and glitter face painting for kids and guests.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>['Professional Entertainment Premium Care Option 2 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Tattoo Artist &amp; Face Painting for Events procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>['Complete Entertainment Premium Care Option 2 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Tattoo Artist &amp; Face Painting for Events procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Entertainment Premium Care Option 2 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 120 minutes.', 'question': 'How long does Tattoo Artist &amp; Face Painting for Events take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>c697f583-d431-5886-aeeb-3d6d3f61300d</t>
+          <t>df202201-6da5-548a-810d-888b497344c3</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1383,47 +1383,47 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management Premium Care Option 11</t>
+          <t>Corporate Conference &amp; Seminar Manager</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>3099</v>
+        <v>8999</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Specialized high-end Event Planning &amp; Management service tailored to specific client needs with extended guarantee.</t>
+          <t>Managing delegate registration badges, AV mic testing, presentation clickers, and tea break logistics.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>['Professional Event Planning &amp; Management Premium Care Option 11 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Corporate Conference &amp; Seminar Manager procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>['Complete Event Planning &amp; Management Premium Care Option 11 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Corporate Conference &amp; Seminar Manager procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Event Planning &amp; Management Premium Care Option 11 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 360 minutes.', 'question': 'How long does Corporate Conference &amp; Seminar Manager take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>cbb9fb78-4d59-5462-913c-eded1c14fc49</t>
+          <t>c697f583-d431-5886-aeeb-3d6d3f61300d</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1438,47 +1438,47 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management Premium Care Option 12</t>
+          <t>End-to-End Birthday Party Coordinator</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>3199</v>
+        <v>4999</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Specialized high-end Event Planning &amp; Management service tailored to specific client needs with extended guarantee.</t>
+          <t>Dedicated event coordinator managing cake arrival, games, anchor, and venue schedule without stress.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>['Professional Event Planning &amp; Management Premium Care Option 12 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional End-to-End Birthday Party Coordinator procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>['Complete Event Planning &amp; Management Premium Care Option 12 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete End-to-End Birthday Party Coordinator procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Event Planning &amp; Management Premium Care Option 12 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 300 minutes.', 'question': 'How long does End-to-End Birthday Party Coordinator take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>df202201-6da5-548a-810d-888b497344c3</t>
+          <t>cbb9fb78-4d59-5462-913c-eded1c14fc49</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1493,40 +1493,40 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Event Planning &amp; Management Premium Care Option 16</t>
+          <t>Pre-Wedding Sangeet &amp; Reception Planner</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>3599</v>
+        <v>14999</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Specialized high-end Event Planning &amp; Management service tailored to specific client needs with extended guarantee.</t>
+          <t>Complete vendor coordination, stage rehearsal schedules, guest escorting, and timeline management.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>['Professional Event Planning &amp; Management Premium Care Option 16 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Pre-Wedding Sangeet &amp; Reception Planner procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>['Complete Event Planning &amp; Management Premium Care Option 16 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Pre-Wedding Sangeet &amp; Reception Planner procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Event Planning &amp; Management Premium Care Option 16 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 480 minutes.', 'question': 'How long does Pre-Wedding Sangeet &amp; Reception Planner take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
@@ -1973,7 +1973,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>bb48e569-a6da-51f5-b3dc-d87f1695b9ca</t>
+          <t>7130a8ad-6e19-53a6-ac85-8f264051dc78</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1988,47 +1988,47 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Premium Care Option 10</t>
+          <t>4K Cinematic Drone Aerial Video Shoot</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>2999</v>
+        <v>4499</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Specialized high-end Photography &amp; Videography service tailored to specific client needs with extended guarantee.</t>
+          <t>FAA/DGCA certified drone pilot capturing majestic top-down cinematic venue perspectives.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>['Professional Photography &amp; Videography Premium Care Option 10 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional 4K Cinematic Drone Aerial Video Shoot procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>['Complete Photography &amp; Videography Premium Care Option 10 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete 4K Cinematic Drone Aerial Video Shoot procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Photography &amp; Videography Premium Care Option 10 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 120 minutes.', 'question': 'How long does 4K Cinematic Drone Aerial Video Shoot take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>fa960fc9-d8f1-5998-8e4b-c1102937d532</t>
+          <t>bb48e569-a6da-51f5-b3dc-d87f1695b9ca</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2043,47 +2043,47 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Premium Care Option 21</t>
+          <t>Instant Photo Booth with Quirky Props &amp; Prints</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>4099</v>
+        <v>5999</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Specialized high-end Photography &amp; Videography service tailored to specific client needs with extended guarantee.</t>
+          <t>On-the-spot magnetic photo strip printing with funny sunglasses, hats, and customized branded frame.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>['Professional Photography &amp; Videography Premium Care Option 21 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Instant Photo Booth with Quirky Props &amp; Prints procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>['Complete Photography &amp; Videography Premium Care Option 21 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Instant Photo Booth with Quirky Props &amp; Prints procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Photography &amp; Videography Premium Care Option 21 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 180 minutes.', 'question': 'How long does Instant Photo Booth with Quirky Props &amp; Prints take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>7130a8ad-6e19-53a6-ac85-8f264051dc78</t>
+          <t>fa960fc9-d8f1-5998-8e4b-c1102937d532</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2098,40 +2098,40 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Photography &amp; Videography Premium Care Option 3</t>
+          <t>Short-Form Social Media Reels Creator</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>2299</v>
+        <v>3499</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Specialized high-end Photography &amp; Videography service tailored to specific client needs with extended guarantee.</t>
+          <t>Vertical format shooting and same-day edited Instagram Reels highlighting event moments.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>['Professional Photography &amp; Videography Premium Care Option 3 procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
+          <t>['Professional Short-Form Social Media Reels Creator procedure', 'Certified &amp; background-verified specialists', 'High-grade safety &amp; sanitized tools', '100% satisfaction guarantee', 'Transparent pricing with zero hidden charges']</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>['Complete Photography &amp; Videography Premium Care Option 3 procedure', 'Standard tools and supplies included', 'Post-service inspection and cleanup', 'Expert consultation and advice']</t>
+          <t>['Complete Short-Form Social Media Reels Creator procedure', 'Standard supplies and equipment', 'Post-service cleanup and inspection', 'Expert guidance and aftercare tips']</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>['Structural heavy modifications', 'Spare hardware unless explicitly requested']</t>
+          <t>['Spare parts or structural replacement unless quoted', 'Hazardous materials']</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>[{'answer': 'The session typically takes around 60 minutes.', 'question': 'How long does Photography &amp; Videography Premium Care Option 3 take?'}, {'answer': 'Yes, strictly industry-approved and sanitized before every appointment.', 'question': 'Are the tools and products safe?'}]</t>
+          <t>[{'answer': 'Typically takes around 150 minutes.', 'question': 'How long does Short-Form Social Media Reels Creator take?'}, {'answer': 'Yes, exact upfront pricing with zero hidden charges.', 'question': 'Is the pricing transparent?'}]</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>7-day service warranty on workmanship</t>
+          <t>7-day service satisfaction warranty</t>
         </is>
       </c>
     </row>

</xml_diff>